<commit_message>
Pull real weather from Open-Meteo instead of a manual sheet
Unlike sensor readings, weather is public data — no reason to make
someone at the finca retype a forecast by hand. climaApi.js fetches
current conditions + hourly outlook from Open-Meteo (free, no API
key) for the finca's coordinates (6°32'22"N 74°37'49"W) and feeds
the same renderPronostico() the sheet-based version used, so the
Clima page needed no markup changes. Also computes a naive
"ventana recomendada" by finding the longest low-rain-probability
stretch in the next 16 hours.

Replaces the just-added sheetPronostico.js, which required two more
manually-maintained sheet tabs for data that's actually automatable.

Refreshes on load, every 15 min, and on tab focus, same pattern as
sensor sync. Falls back to the page's static content if the API is
unreachable.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sensores-finca.xlsx
+++ b/sensores-finca.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -566,16 +566,16 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Lote B · Mango</t>
+          <t>Lote A · Cacao</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Humedad</t>
+          <t>Humedad de suelo</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
@@ -584,7 +584,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>alerta</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -596,20 +596,20 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Lote C · Café</t>
+          <t>Lote A · Cacao</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Humedad</t>
+          <t>Temperatura</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Lote D · Cacao</t>
+          <t>Lote B · Mango</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>aviso</t>
+          <t>alerta</t>
         </is>
       </c>
     </row>
@@ -656,25 +656,25 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Vivero</t>
+          <t>Lote B · Mango</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Temperatura</t>
+          <t>Humedad de suelo</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>alerta</t>
         </is>
       </c>
     </row>
@@ -686,75 +686,315 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
+          <t>Lote B · Mango</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Temperatura</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>aviso</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>S-07</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Lote C · Café</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Humedad</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>S-08</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Lote C · Café</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Humedad de suelo</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>S-09</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Lote C · Café</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Temperatura</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>S-10</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Lote D · Cacao</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Humedad</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>aviso</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>S-11</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Lote D · Cacao</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Humedad de suelo</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>aviso</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>S-12</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Lote D · Cacao</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Temperatura</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>S-13</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Vivero</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Temperatura</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>S-14</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
           <t>Zona hídrica</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Caudal riego</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>l/m</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>sin señal</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n"/>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -772,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -833,43 +1073,50 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Vivero, Zona hídrica). 'tipo' es lo que mide (Humedad, Temperatura, etc).</t>
+          <t xml:space="preserve">   Vivero, Zona hídrica). Cada Lote tiene 3 filas, una por 'tipo': Humedad,</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>6. Para agregar un sensor nuevo, usa una fila vacía y completa las 6 columnas.</t>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Humedad de suelo y Temperatura.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
+          <t>6. Para agregar un sensor nuevo, usa una fila vacía y completa las 6 columnas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
           <t>7. No hace falta guardar nada especial — Google Sheets guarda solo.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>El sitio web lee esta hoja automáticamente cada pocos minutos.</t>
-        </is>
-      </c>
+      <c r="A13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Si algo se ve raro en la web, revisa que 'estado' tenga exactamente una de esas</t>
+          <t>El sitio web lee esta hoja automáticamente cada pocos minutos.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Si algo se ve raro en la web, revisa que 'estado' tenga exactamente una de esas</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>cuatro palabras y que 'valor' sea un número.</t>
         </is>

</xml_diff>